<commit_message>
Extend template to 500 rows
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KoEmo_template.xlsx
+++ b/docs/KoEmo_template.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F105"/>
+  <dimension ref="A1:F505"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="6" min="1" max="1"/>
@@ -1630,9 +1630,2009 @@
       <c r="E105" s="3" t="n"/>
       <c r="F105" s="3" t="n"/>
     </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="n">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="n">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="n">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="n">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="n">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="n">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="n">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="n">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="n">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="n">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="n">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="n">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="n">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="n">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="n">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="n">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="n">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="n">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="n">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="n">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="n">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="n">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="n">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="n">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="n">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="n">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="n">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="n">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="n">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="n">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="n">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="n">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="n">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="n">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="n">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="n">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="n">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="n">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="n">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="n">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="n">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="n">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="n">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="n">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="n">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="n">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="n">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="n">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="n">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="n">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="n">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="n">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="n">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="n">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="n">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="n">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="n">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="n">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="n">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="n">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="n">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="n">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="n">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="n">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="n">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="n">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="n">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="n">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="n">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="n">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="n">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="n">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="n">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="n">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="n">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="n">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="n">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="n">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="n">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="n">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="n">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="n">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="n">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="n">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="n">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="n">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="n">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="n">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="n">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="n">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="n">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="n">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="n">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="n">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="n">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="n">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="n">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="n">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="n">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="n">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="n">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="n">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="n">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="n">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="n">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="n">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="n">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="n">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="n">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="n">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="n">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="n">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="n">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="n">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="n">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="n">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="n">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="n">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="n">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="n">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="n">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="n">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="n">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="n">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="n">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="n">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="n">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="n">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="n">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="n">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="n">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="n">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="n">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="n">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="n">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="n">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="n">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="n">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="n">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="n">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="n">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="n">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="n">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="n">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="n">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="n">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="n">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="n">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="n">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="n">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="n">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="n">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="n">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="n">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="n">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="n">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="n">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="n">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="n">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="n">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="n">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="n">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="n">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="n">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="n">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="n">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="n">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="n">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="n">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="n">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="n">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="n">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="n">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="n">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="n">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="n">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="n">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="n">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="n">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="n">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="n">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="n">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="n">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="n">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="n">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="n">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="n">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="n">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="n">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="n">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="n">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="n">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="n">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="n">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="n">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="n">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="n">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="n">
+        <v>500</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B6:B105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="도메인 선택 오류" error="5가지 도메인 중에서 선택해 주세요." promptTitle="도메인" prompt="도메인을 선택하세요." type="list">
+    <dataValidation sqref="B6:B505" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="도메인 선택 오류" error="5가지 도메인 중에서 선택해 주세요." promptTitle="도메인" prompt="도메인을 선택하세요." type="list">
       <formula1>"감각 표현,감정 표현,판단 표현,감상 표현,상징 표현"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Final review fixes: remove 5th XLSX example, clarify guidelines
- Remove 5th example row (시원하다) from XLSX template
- Fix XLSX 정답 header to match guideline (유의어군 중 택1)
- Clarify 문체/시제 통일 with concrete reference to example table
- Add example for "너무 뻔하게 틀린 상황" to make it understandable

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KoEmo_template.xlsx
+++ b/docs/KoEmo_template.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F506"/>
+  <dimension ref="A1:F505"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="11" min="1" max="1"/>
@@ -500,7 +500,7 @@
       </c>
       <c r="E1" s="9" t="inlineStr">
         <is>
-          <t>정답 (단어군 중 하나 선택)</t>
+          <t>정답 (유의어군 중 택1)</t>
         </is>
       </c>
       <c r="F1" s="9" t="inlineStr">
@@ -638,2734 +638,2702 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>(예시)</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>감각 표현</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>미각</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>맵다, 얼큰하다, 알싸하다, 시원하다</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>시원하다</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>김치찌개에 청양고추를 넣었더니 국물이 [정답].</t>
-        </is>
-      </c>
+      <c r="A6" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B7" s="11" t="n"/>
       <c r="C7" s="11" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B8" s="11" t="n"/>
       <c r="C8" s="11" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B9" s="11" t="n"/>
       <c r="C9" s="11" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B10" s="11" t="n"/>
       <c r="C10" s="11" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B11" s="11" t="n"/>
       <c r="C11" s="11" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B12" s="11" t="n"/>
       <c r="C12" s="11" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B13" s="11" t="n"/>
       <c r="C13" s="11" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B14" s="11" t="n"/>
       <c r="C14" s="11" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B15" s="11" t="n"/>
       <c r="C15" s="11" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B16" s="11" t="n"/>
       <c r="C16" s="11" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B17" s="11" t="n"/>
       <c r="C17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B18" s="11" t="n"/>
       <c r="C18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="11" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B19" s="11" t="n"/>
       <c r="C19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="11" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B20" s="11" t="n"/>
       <c r="C20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="11" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B21" s="11" t="n"/>
       <c r="C21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="11" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B22" s="11" t="n"/>
       <c r="C22" s="11" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="11" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B23" s="11" t="n"/>
       <c r="C23" s="11" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="11" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B24" s="11" t="n"/>
       <c r="C24" s="11" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="11" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B25" s="11" t="n"/>
       <c r="C25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B26" s="11" t="n"/>
       <c r="C26" s="11" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="11" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B27" s="11" t="n"/>
       <c r="C27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="11" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B28" s="11" t="n"/>
       <c r="C28" s="11" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="11" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B29" s="11" t="n"/>
       <c r="C29" s="11" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="11" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B30" s="11" t="n"/>
       <c r="C30" s="11" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="11" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B31" s="11" t="n"/>
       <c r="C31" s="11" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="11" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B32" s="11" t="n"/>
       <c r="C32" s="11" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="11" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B33" s="11" t="n"/>
       <c r="C33" s="11" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="11" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B34" s="11" t="n"/>
       <c r="C34" s="11" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="11" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B35" s="11" t="n"/>
       <c r="C35" s="11" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B36" s="11" t="n"/>
       <c r="C36" s="11" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B37" s="11" t="n"/>
       <c r="C37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="11" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B38" s="11" t="n"/>
       <c r="C38" s="11" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="11" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B39" s="11" t="n"/>
       <c r="C39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="11" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B40" s="11" t="n"/>
       <c r="C40" s="11" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="11" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B41" s="11" t="n"/>
       <c r="C41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="11" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B42" s="11" t="n"/>
       <c r="C42" s="11" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="11" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B43" s="11" t="n"/>
       <c r="C43" s="11" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="11" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B44" s="11" t="n"/>
       <c r="C44" s="11" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="11" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B45" s="11" t="n"/>
       <c r="C45" s="11" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="11" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B46" s="11" t="n"/>
       <c r="C46" s="11" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="11" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B47" s="11" t="n"/>
       <c r="C47" s="11" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="11" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B48" s="11" t="n"/>
       <c r="C48" s="11" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="11" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B49" s="11" t="n"/>
       <c r="C49" s="11" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="11" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B50" s="11" t="n"/>
       <c r="C50" s="11" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="11" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B51" s="11" t="n"/>
       <c r="C51" s="11" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B52" s="11" t="n"/>
       <c r="C52" s="11" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B53" s="11" t="n"/>
       <c r="C53" s="11" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="11" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B54" s="11" t="n"/>
       <c r="C54" s="11" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B55" s="11" t="n"/>
       <c r="C55" s="11" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B56" s="11" t="n"/>
       <c r="C56" s="11" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B57" s="11" t="n"/>
       <c r="C57" s="11" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B58" s="11" t="n"/>
       <c r="C58" s="11" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="11" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B59" s="11" t="n"/>
       <c r="C59" s="11" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B60" s="11" t="n"/>
       <c r="C60" s="11" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B61" s="11" t="n"/>
       <c r="C61" s="11" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B62" s="11" t="n"/>
       <c r="C62" s="11" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B63" s="11" t="n"/>
       <c r="C63" s="11" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="11" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B64" s="11" t="n"/>
       <c r="C64" s="11" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="11" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B65" s="11" t="n"/>
       <c r="C65" s="11" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="11" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B66" s="11" t="n"/>
       <c r="C66" s="11" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="11" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B67" s="11" t="n"/>
       <c r="C67" s="11" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="11" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B68" s="11" t="n"/>
       <c r="C68" s="11" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="11" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B69" s="11" t="n"/>
       <c r="C69" s="11" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="11" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B70" s="11" t="n"/>
       <c r="C70" s="11" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="11" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B71" s="11" t="n"/>
       <c r="C71" s="11" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="11" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B72" s="11" t="n"/>
       <c r="C72" s="11" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="11" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B73" s="11" t="n"/>
       <c r="C73" s="11" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="11" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B74" s="11" t="n"/>
       <c r="C74" s="11" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="11" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B75" s="11" t="n"/>
       <c r="C75" s="11" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="11" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B76" s="11" t="n"/>
       <c r="C76" s="11" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="11" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B77" s="11" t="n"/>
       <c r="C77" s="11" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="11" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B78" s="11" t="n"/>
       <c r="C78" s="11" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="11" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B79" s="11" t="n"/>
       <c r="C79" s="11" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="11" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B80" s="11" t="n"/>
       <c r="C80" s="11" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="11" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B81" s="11" t="n"/>
       <c r="C81" s="11" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="11" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B82" s="11" t="n"/>
       <c r="C82" s="11" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="11" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B83" s="11" t="n"/>
       <c r="C83" s="11" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="11" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B84" s="11" t="n"/>
       <c r="C84" s="11" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="11" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B85" s="11" t="n"/>
       <c r="C85" s="11" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="11" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B86" s="11" t="n"/>
       <c r="C86" s="11" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="11" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B87" s="11" t="n"/>
       <c r="C87" s="11" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="11" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B88" s="11" t="n"/>
       <c r="C88" s="11" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="11" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B89" s="11" t="n"/>
       <c r="C89" s="11" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="11" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B90" s="11" t="n"/>
       <c r="C90" s="11" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="11" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B91" s="11" t="n"/>
       <c r="C91" s="11" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="11" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B92" s="11" t="n"/>
       <c r="C92" s="11" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="11" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B93" s="11" t="n"/>
       <c r="C93" s="11" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="11" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B94" s="11" t="n"/>
       <c r="C94" s="11" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="11" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B95" s="11" t="n"/>
       <c r="C95" s="11" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="11" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B96" s="11" t="n"/>
       <c r="C96" s="11" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="11" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B97" s="11" t="n"/>
       <c r="C97" s="11" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="11" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B98" s="11" t="n"/>
       <c r="C98" s="11" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="11" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B99" s="11" t="n"/>
       <c r="C99" s="11" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="11" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B100" s="11" t="n"/>
       <c r="C100" s="11" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="11" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B101" s="11" t="n"/>
       <c r="C101" s="11" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="11" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B102" s="11" t="n"/>
       <c r="C102" s="11" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="11" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B103" s="11" t="n"/>
       <c r="C103" s="11" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="11" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B104" s="11" t="n"/>
       <c r="C104" s="11" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="11" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B105" s="11" t="n"/>
       <c r="C105" s="11" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="11" t="n">
-        <v>100</v>
-      </c>
-      <c r="B106" s="11" t="n"/>
-      <c r="C106" s="11" t="n"/>
+      <c r="A106" s="4" t="n">
+        <v>101</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="4" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="4" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="4" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="4" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="4" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="4" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="4" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="4" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="4" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="4" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="4" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="4" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="4" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="4" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="4" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="4" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="4" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="4" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="4" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="4" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="4" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="4" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="4" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="4" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="4" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="4" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="4" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="4" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="4" t="n">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="4" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="4" t="n">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="4" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="n">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="4" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="4" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="4" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="4" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="4" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="4" t="n">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="4" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="4" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="4" t="n">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="4" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="4" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="4" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="4" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="4" t="n">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="4" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="4" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="4" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="4" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="4" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="4" t="n">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="4" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="4" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="4" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="4" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="4" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="4" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="4" t="n">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="4" t="n">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="4" t="n">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="4" t="n">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="4" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="4" t="n">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="4" t="n">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="4" t="n">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="4" t="n">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="4" t="n">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="4" t="n">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="4" t="n">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="4" t="n">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="4" t="n">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="4" t="n">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="4" t="n">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="4" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="4" t="n">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="4" t="n">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="4" t="n">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="4" t="n">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="4" t="n">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="4" t="n">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="4" t="n">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="4" t="n">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="4" t="n">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="4" t="n">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="4" t="n">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="4" t="n">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="4" t="n">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="4" t="n">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="4" t="n">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="4" t="n">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="4" t="n">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="4" t="n">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="4" t="n">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="4" t="n">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="4" t="n">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="4" t="n">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="4" t="n">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="4" t="n">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="4" t="n">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="4" t="n">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="4" t="n">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="4" t="n">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="4" t="n">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="4" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="4" t="n">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="4" t="n">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="4" t="n">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="4" t="n">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="4" t="n">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="4" t="n">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="4" t="n">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="4" t="n">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="4" t="n">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="4" t="n">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="4" t="n">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="4" t="n">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="4" t="n">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="4" t="n">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="4" t="n">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="4" t="n">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="4" t="n">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="4" t="n">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="4" t="n">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="4" t="n">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="4" t="n">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="4" t="n">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="4" t="n">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="4" t="n">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="4" t="n">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="4" t="n">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="4" t="n">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="4" t="n">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="4" t="n">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="4" t="n">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="4" t="n">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="4" t="n">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="4" t="n">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="4" t="n">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="4" t="n">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="4" t="n">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="4" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="4" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="4" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="4" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="4" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="4" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="4" t="n">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="4" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="4" t="n">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="4" t="n">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="4" t="n">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="4" t="n">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="4" t="n">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="4" t="n">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="4" t="n">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="4" t="n">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="4" t="n">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="4" t="n">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="4" t="n">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="4" t="n">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="4" t="n">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="4" t="n">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="4" t="n">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="4" t="n">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="4" t="n">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="4" t="n">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="4" t="n">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="4" t="n">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="4" t="n">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="4" t="n">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" s="4" t="n">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="4" t="n">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" s="4" t="n">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="4" t="n">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="4" t="n">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="4" t="n">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="4" t="n">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" s="4" t="n">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="4" t="n">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="4" t="n">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="4" t="n">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" s="4" t="n">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" s="4" t="n">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" s="4" t="n">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="4" t="n">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" s="4" t="n">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" s="4" t="n">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" s="4" t="n">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" s="4" t="n">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" s="4" t="n">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" s="4" t="n">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" s="4" t="n">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" s="4" t="n">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" s="4" t="n">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" s="4" t="n">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" s="4" t="n">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="4" t="n">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" s="4" t="n">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="4" t="n">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="4" t="n">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="4" t="n">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="4" t="n">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="4" t="n">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="4" t="n">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="4" t="n">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="4" t="n">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="4" t="n">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="4" t="n">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="4" t="n">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" s="4" t="n">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" s="4" t="n">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="4" t="n">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" s="4" t="n">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" s="4" t="n">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" s="4" t="n">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" s="4" t="n">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="4" t="n">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" s="4" t="n">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="4" t="n">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" s="4" t="n">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="4" t="n">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="4" t="n">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="4" t="n">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="4" t="n">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" s="4" t="n">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="4" t="n">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="4" t="n">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="4" t="n">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" s="4" t="n">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" s="4" t="n">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" s="4" t="n">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="4" t="n">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" s="4" t="n">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" s="4" t="n">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" s="4" t="n">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" s="4" t="n">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="4" t="n">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" s="4" t="n">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" s="4" t="n">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" s="4" t="n">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" s="4" t="n">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" s="4" t="n">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" s="4" t="n">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" s="4" t="n">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" s="4" t="n">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" s="4" t="n">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" s="4" t="n">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" s="4" t="n">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" s="4" t="n">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" s="4" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" s="4" t="n">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" s="4" t="n">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" s="4" t="n">
-        <v>379</v>
+        <v>380</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" s="4" t="n">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" s="4" t="n">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" s="4" t="n">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="389">
       <c r="A389" s="4" t="n">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" s="4" t="n">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="391">
       <c r="A391" s="4" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="392">
       <c r="A392" s="4" t="n">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" s="4" t="n">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" s="4" t="n">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" s="4" t="n">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" s="4" t="n">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" s="4" t="n">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" s="4" t="n">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" s="4" t="n">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" s="4" t="n">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" s="4" t="n">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" s="4" t="n">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" s="4" t="n">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" s="4" t="n">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" s="4" t="n">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" s="4" t="n">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" s="4" t="n">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" s="4" t="n">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" s="4" t="n">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" s="4" t="n">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="411">
       <c r="A411" s="4" t="n">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" s="4" t="n">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="413">
       <c r="A413" s="4" t="n">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="414">
       <c r="A414" s="4" t="n">
-        <v>408</v>
+        <v>409</v>
       </c>
     </row>
     <row r="415">
       <c r="A415" s="4" t="n">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="416">
       <c r="A416" s="4" t="n">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="417">
       <c r="A417" s="4" t="n">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="4" t="n">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" s="4" t="n">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="4" t="n">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" s="4" t="n">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="4" t="n">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="4" t="n">
-        <v>417</v>
+        <v>418</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="4" t="n">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="4" t="n">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="4" t="n">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="4" t="n">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="4" t="n">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="4" t="n">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="4" t="n">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="4" t="n">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="4" t="n">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="4" t="n">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="4" t="n">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="4" t="n">
-        <v>429</v>
+        <v>430</v>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="4" t="n">
-        <v>430</v>
+        <v>431</v>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="4" t="n">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="4" t="n">
-        <v>432</v>
+        <v>433</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="4" t="n">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="4" t="n">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="4" t="n">
-        <v>435</v>
+        <v>436</v>
       </c>
     </row>
     <row r="442">
       <c r="A442" s="4" t="n">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="4" t="n">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="4" t="n">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="4" t="n">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="4" t="n">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="4" t="n">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="4" t="n">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="4" t="n">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="4" t="n">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="4" t="n">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="4" t="n">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="4" t="n">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="4" t="n">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="4" t="n">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="456">
       <c r="A456" s="4" t="n">
-        <v>450</v>
+        <v>451</v>
       </c>
     </row>
     <row r="457">
       <c r="A457" s="4" t="n">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="458">
       <c r="A458" s="4" t="n">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="459">
       <c r="A459" s="4" t="n">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="460">
       <c r="A460" s="4" t="n">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
     <row r="461">
       <c r="A461" s="4" t="n">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
     <row r="462">
       <c r="A462" s="4" t="n">
-        <v>456</v>
+        <v>457</v>
       </c>
     </row>
     <row r="463">
       <c r="A463" s="4" t="n">
-        <v>457</v>
+        <v>458</v>
       </c>
     </row>
     <row r="464">
       <c r="A464" s="4" t="n">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="465">
       <c r="A465" s="4" t="n">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="466">
       <c r="A466" s="4" t="n">
-        <v>460</v>
+        <v>461</v>
       </c>
     </row>
     <row r="467">
       <c r="A467" s="4" t="n">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="468">
       <c r="A468" s="4" t="n">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="469">
       <c r="A469" s="4" t="n">
-        <v>463</v>
+        <v>464</v>
       </c>
     </row>
     <row r="470">
       <c r="A470" s="4" t="n">
-        <v>464</v>
+        <v>465</v>
       </c>
     </row>
     <row r="471">
       <c r="A471" s="4" t="n">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="472">
       <c r="A472" s="4" t="n">
-        <v>466</v>
+        <v>467</v>
       </c>
     </row>
     <row r="473">
       <c r="A473" s="4" t="n">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="474">
       <c r="A474" s="4" t="n">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="475">
       <c r="A475" s="4" t="n">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="476">
       <c r="A476" s="4" t="n">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
     <row r="477">
       <c r="A477" s="4" t="n">
-        <v>471</v>
+        <v>472</v>
       </c>
     </row>
     <row r="478">
       <c r="A478" s="4" t="n">
-        <v>472</v>
+        <v>473</v>
       </c>
     </row>
     <row r="479">
       <c r="A479" s="4" t="n">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="480">
       <c r="A480" s="4" t="n">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="481">
       <c r="A481" s="4" t="n">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="482">
       <c r="A482" s="4" t="n">
-        <v>476</v>
+        <v>477</v>
       </c>
     </row>
     <row r="483">
       <c r="A483" s="4" t="n">
-        <v>477</v>
+        <v>478</v>
       </c>
     </row>
     <row r="484">
       <c r="A484" s="4" t="n">
-        <v>478</v>
+        <v>479</v>
       </c>
     </row>
     <row r="485">
       <c r="A485" s="4" t="n">
-        <v>479</v>
+        <v>480</v>
       </c>
     </row>
     <row r="486">
       <c r="A486" s="4" t="n">
-        <v>480</v>
+        <v>481</v>
       </c>
     </row>
     <row r="487">
       <c r="A487" s="4" t="n">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="488">
       <c r="A488" s="4" t="n">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
     <row r="489">
       <c r="A489" s="4" t="n">
-        <v>483</v>
+        <v>484</v>
       </c>
     </row>
     <row r="490">
       <c r="A490" s="4" t="n">
-        <v>484</v>
+        <v>485</v>
       </c>
     </row>
     <row r="491">
       <c r="A491" s="4" t="n">
-        <v>485</v>
+        <v>486</v>
       </c>
     </row>
     <row r="492">
       <c r="A492" s="4" t="n">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row r="493">
       <c r="A493" s="4" t="n">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="494">
       <c r="A494" s="4" t="n">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="495">
       <c r="A495" s="4" t="n">
-        <v>489</v>
+        <v>490</v>
       </c>
     </row>
     <row r="496">
       <c r="A496" s="4" t="n">
-        <v>490</v>
+        <v>491</v>
       </c>
     </row>
     <row r="497">
       <c r="A497" s="4" t="n">
-        <v>491</v>
+        <v>492</v>
       </c>
     </row>
     <row r="498">
       <c r="A498" s="4" t="n">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="499">
       <c r="A499" s="4" t="n">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="500">
       <c r="A500" s="4" t="n">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="501">
       <c r="A501" s="4" t="n">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="502">
       <c r="A502" s="4" t="n">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="503">
       <c r="A503" s="4" t="n">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row r="504">
       <c r="A504" s="4" t="n">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="505">
       <c r="A505" s="4" t="n">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="506">
-      <c r="A506" s="4" t="n">
         <v>500</v>
       </c>
     </row>

</xml_diff>